<commit_message>
fix: regenerate test_4_ce_students.xlsx as fee records for SMS testing
</commit_message>
<xml_diff>
--- a/backend/excel-files/test_4_ce_students.xlsx
+++ b/backend/excel-files/test_4_ce_students.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Students" sheetId="1" r:id="rId1"/>
+    <sheet name="Fees" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,151 +397,119 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:F5"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="18.83203125" customWidth="1"/>
-    <col min="3" max="3" width="35.83203125" customWidth="1"/>
-    <col min="4" max="4" width="45.83203125" customWidth="1"/>
-    <col min="5" max="5" width="40.83203125" customWidth="1"/>
+    <col min="2" max="2" width="25.83203125" customWidth="1"/>
+    <col min="3" max="3" width="15.83203125" customWidth="1"/>
+    <col min="4" max="4" width="15.83203125" customWidth="1"/>
+    <col min="5" max="5" width="15.83203125" customWidth="1"/>
     <col min="6" max="6" width="12.83203125" customWidth="1"/>
-    <col min="7" max="7" width="15.83203125" customWidth="1"/>
-    <col min="8" max="8" width="15.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Name</v>
+        <v>Index Number</v>
       </c>
       <c r="B1" t="str">
-        <v>Index Number</v>
+        <v>Student Name</v>
       </c>
       <c r="C1" t="str">
-        <v>Email</v>
+        <v>Total Amount</v>
       </c>
       <c r="D1" t="str">
-        <v>Programme</v>
+        <v>Amount Paid</v>
       </c>
       <c r="E1" t="str">
-        <v>Department</v>
+        <v>Academic Year</v>
       </c>
       <c r="F1" t="str">
-        <v>Cohort</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Academic Year</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Phone Number</v>
+        <v>Semester</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
+        <v>UMaT/PG/0003/22</v>
+      </c>
+      <c r="B2" t="str">
         <v>Mensah Agyei</v>
       </c>
-      <c r="B2" t="str">
-        <v>UMaT/PG/0003/22</v>
-      </c>
-      <c r="C2" t="str">
-        <v>mensah.agyei3@umat.edu.gh</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Computer Science and Engineering MPhil</v>
+      <c r="C2">
+        <v>8000</v>
+      </c>
+      <c r="D2">
+        <v>5000</v>
       </c>
       <c r="E2" t="str">
-        <v>Computer Science and Engineering</v>
+        <v>2024/2025</v>
       </c>
       <c r="F2" t="str">
-        <v>July</v>
-      </c>
-      <c r="G2" t="str">
-        <v>2024/2025</v>
-      </c>
-      <c r="H2" t="str">
-        <v>0531399032</v>
+        <v>First</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
+        <v>UMaT/PG/0008/22</v>
+      </c>
+      <c r="B3" t="str">
         <v>Kwabena Ofori</v>
       </c>
-      <c r="B3" t="str">
-        <v>UMaT/PG/0008/22</v>
-      </c>
-      <c r="C3" t="str">
-        <v>kwabena.ofori8@umat.edu.gh</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Computer Science and Engineering MPhil</v>
+      <c r="C3">
+        <v>8000</v>
+      </c>
+      <c r="D3">
+        <v>5000</v>
       </c>
       <c r="E3" t="str">
-        <v>Computer Science and Engineering</v>
+        <v>2024/2025</v>
       </c>
       <c r="F3" t="str">
-        <v>January</v>
-      </c>
-      <c r="G3" t="str">
-        <v>2024/2025</v>
-      </c>
-      <c r="H3" t="str">
-        <v>0548329408</v>
+        <v>First</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
+        <v>UMaT/PG/0009/22</v>
+      </c>
+      <c r="B4" t="str">
         <v>Panyin Darko</v>
       </c>
-      <c r="B4" t="str">
-        <v>UMaT/PG/0009/22</v>
-      </c>
-      <c r="C4" t="str">
-        <v>panyin.darko9@umat.edu.gh</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Computer Science and Engineering MSc</v>
+      <c r="C4">
+        <v>8000</v>
+      </c>
+      <c r="D4">
+        <v>5000</v>
       </c>
       <c r="E4" t="str">
-        <v>Computer Science and Engineering</v>
+        <v>2024/2025</v>
       </c>
       <c r="F4" t="str">
-        <v>July</v>
-      </c>
-      <c r="G4" t="str">
-        <v>2024/2025</v>
-      </c>
-      <c r="H4" t="str">
-        <v>0592826345</v>
+        <v>First</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
+        <v>UMaT/PG/0015/22</v>
+      </c>
+      <c r="B5" t="str">
         <v>Ebo Mensah</v>
       </c>
-      <c r="B5" t="str">
-        <v>UMaT/PG/0015/22</v>
-      </c>
-      <c r="C5" t="str">
-        <v>ebo.mensah15@umat.edu.gh</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Computer Science and Engineering MPhil</v>
+      <c r="C5">
+        <v>8000</v>
+      </c>
+      <c r="D5">
+        <v>5000</v>
       </c>
       <c r="E5" t="str">
-        <v>Computer Science and Engineering</v>
+        <v>2024/2025</v>
       </c>
       <c r="F5" t="str">
-        <v>January</v>
-      </c>
-      <c r="G5" t="str">
-        <v>2024/2025</v>
-      </c>
-      <c r="H5" t="str">
-        <v>0595799116</v>
+        <v>First</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>